<commit_message>
Update UI and server logic and refresh base data
</commit_message>
<xml_diff>
--- a/data/Base_data.xlsx
+++ b/data/Base_data.xlsx
@@ -716,7 +716,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
@@ -928,6 +928,29 @@
         <v>46006</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>Auto: ändring bonus_grund i Konsulter-tabell</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BN-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CONS-010</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>6</v>
+      </c>
+      <c r="D10" s="2">
+        <v>46108</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Auto: ändring bonus_grund i Konsulter-tabell</t>
         </is>
@@ -3153,7 +3176,7 @@
         <v>50000</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I11" s="2">
         <v>46023</v>

</xml_diff>

<commit_message>
Add filtering in bonus report tab
</commit_message>
<xml_diff>
--- a/data/Base_data.xlsx
+++ b/data/Base_data.xlsx
@@ -368,7 +368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -706,6 +706,33 @@
       <c r="K9" t="inlineStr">
         <is>
           <t>Auto från Kunder (FM-typ Kund)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FM-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mäklare</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MAKL-CUSTOM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CUST-POSTNO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Auto från Kunder (FM-typ Mäklare)</t>
         </is>
       </c>
     </row>
@@ -716,7 +743,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
@@ -951,6 +978,52 @@
         <v>46108</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>Auto: ändring bonus_grund i Konsulter-tabell</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BN-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>8</v>
+      </c>
+      <c r="D11" s="2">
+        <v>46023</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Auto vid ny konsult</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BN-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2">
+        <v>46024</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Auto: ändring bonus_grund i Konsulter-tabell</t>
         </is>
@@ -1357,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="20.7109375" style="2" customWidth="1"/>
@@ -2357,6 +2430,128 @@
         <v>2928</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BR-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>group_bonus</t>
+        </is>
+      </c>
+      <c r="C17" s="2">
+        <v>46054</v>
+      </c>
+      <c r="D17" s="2">
+        <v>46081</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CONS-004</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CUST-POSTNO</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>UPP-012</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>TASK-014</t>
+        </is>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>98</v>
+      </c>
+      <c r="L17" s="2">
+        <v>46113</v>
+      </c>
+      <c r="M17">
+        <v>1100</v>
+      </c>
+      <c r="N17">
+        <v>107800</v>
+      </c>
+      <c r="O17">
+        <v>3234</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BR-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>sales_bonus</t>
+        </is>
+      </c>
+      <c r="C18" s="2">
+        <v>46054</v>
+      </c>
+      <c r="D18" s="2">
+        <v>46081</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CONS-002</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CUST-POSTNO</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UPP-012</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>TASK-014</t>
+        </is>
+      </c>
+      <c r="J18">
+        <v>4</v>
+      </c>
+      <c r="K18">
+        <v>98</v>
+      </c>
+      <c r="L18" s="2">
+        <v>46113</v>
+      </c>
+      <c r="M18">
+        <v>1100</v>
+      </c>
+      <c r="N18">
+        <v>107800</v>
+      </c>
+      <c r="O18">
+        <v>4312</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2364,7 +2559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -2464,7 +2659,7 @@
         </is>
       </c>
       <c r="G3" s="2">
-        <v>46094</v>
+        <v>46037</v>
       </c>
     </row>
     <row r="4">
@@ -2494,7 +2689,7 @@
         </is>
       </c>
       <c r="G4" s="2">
-        <v>46094</v>
+        <v>46037</v>
       </c>
     </row>
     <row r="5">
@@ -2524,7 +2719,42 @@
         </is>
       </c>
       <c r="G5" s="2">
-        <v>46094</v>
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAKL-CUSTOM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Custome</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Culter</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>jon.culter@custom.se</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ska ändras senare</t>
+        </is>
+      </c>
+      <c r="G6" s="2">
+        <v>46037</v>
       </c>
     </row>
   </sheetData>
@@ -2534,7 +2764,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -2809,7 +3039,37 @@
         </is>
       </c>
       <c r="F9" s="2">
-        <v>46376</v>
+        <v>46011</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CUST-POSTNO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Postnord</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Shultz</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>lena.shultz@postnord.se</t>
+        </is>
+      </c>
+      <c r="F10" s="2">
+        <v>46037</v>
       </c>
     </row>
   </sheetData>
@@ -2819,7 +3079,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="9" max="9" width="20.7109375" style="2" customWidth="1"/>
@@ -3182,6 +3442,37 @@
         <v>46023</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Johan</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Strand</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Anställd</t>
+        </is>
+      </c>
+      <c r="E12">
+        <v>50000</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="I12" s="2">
+        <v>46023</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3189,7 +3480,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
@@ -3236,363 +3527,396 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UPP-001</t>
+          <t>UPP-012</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Domus plattformsmigrering</t>
+          <t>Postnord Prisprediktion</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Digital plattformsmigrering</t>
+          <t>Prisanalys och prognos</t>
         </is>
       </c>
       <c r="D2" s="2">
-        <v>45307</v>
+        <v>46054</v>
       </c>
       <c r="E2" s="2">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-POSTNO</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>FM-001</t>
+          <t>FM-009</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UPP-002</t>
+          <t>UPP-011</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Domus Database och BI</t>
+          <t>Nanometer Datakvalitet</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Database och BI-mothernisering</t>
+          <t>Utredning av datakvalitet</t>
         </is>
       </c>
       <c r="D3" s="2">
-        <v>45307</v>
+        <v>46026</v>
       </c>
       <c r="E3" s="2">
         <v>46387</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-NANOME</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FM-001</t>
+          <t>FM-008</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UPP-003</t>
+          <t>UPP-010</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Domus automatisering</t>
+          <t>Baral Azure inloggning</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sistemintegration och automatisering</t>
+          <t>Implementering av inloggning Azure Directory</t>
         </is>
       </c>
       <c r="D4" s="2">
-        <v>45307</v>
+        <v>45935</v>
       </c>
       <c r="E4" s="2">
-        <v>46203</v>
+        <v>46295</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-BARAL</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>FM-001</t>
+          <t>FM-007</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>UPP-004</t>
+          <t>UPP-009</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RSV Data utredning</t>
+          <t>Lansa Kravanalys</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Utredning av tillgängligt data</t>
+          <t>Förstudie och kravanalys</t>
         </is>
       </c>
       <c r="D5" s="2">
-        <v>45453</v>
+        <v>45813</v>
       </c>
       <c r="E5" s="2">
-        <v>46173</v>
+        <v>46203</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-LANSA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>FM-002</t>
+          <t>FM-006</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UPP-005</t>
+          <t>UPP-008</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Avista Kvalitetssäkring</t>
+          <t>Mondo Uppbyggnad av datalagret</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kvalitetssäkring och datarensning</t>
+          <t>Uppbyggnad av datalager för försäljning</t>
         </is>
       </c>
       <c r="D6" s="2">
-        <v>45458</v>
+        <v>45797</v>
       </c>
       <c r="E6" s="2">
-        <v>46387</v>
+        <v>46112</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CUST-AVISTA</t>
+          <t>CUST-MONDO</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>FM-003</t>
+          <t>FM-005</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UPP-006</t>
+          <t>UPP-007</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RSV Database migrering</t>
+          <t>Opus CRM och ERP integration</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Utredning och database migrering</t>
+          <t>Data Integration mellan CRM och ERP sistem</t>
         </is>
       </c>
       <c r="D7" s="2">
         <v>45672</v>
       </c>
       <c r="E7" s="2">
-        <v>46387</v>
+        <v>46203</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-OPUS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>FM-002</t>
+          <t>FM-004</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UPP-007</t>
+          <t>UPP-006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Opus CRM och ERP integration</t>
+          <t>RSV Database migrering</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Data Integration mellan CRM och ERP sistem</t>
+          <t>Utredning och database migrering</t>
         </is>
       </c>
       <c r="D8" s="2">
         <v>45672</v>
       </c>
       <c r="E8" s="2">
-        <v>46203</v>
+        <v>46387</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CUST-OPUS</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>FM-004</t>
+          <t>FM-002</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UPP-008</t>
+          <t>UPP-005</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mondo Uppbyggnad av datalagret</t>
+          <t>Avista Kvalitetssäkring</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Uppbyggnad av datalager för försäljning</t>
+          <t>Kvalitetssäkring och datarensning</t>
         </is>
       </c>
       <c r="D9" s="2">
-        <v>45797</v>
+        <v>45458</v>
       </c>
       <c r="E9" s="2">
-        <v>46112</v>
+        <v>46387</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CUST-MONDO</t>
+          <t>CUST-AVISTA</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>FM-005</t>
+          <t>FM-003</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UPP-009</t>
+          <t>UPP-004</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lansa Kravanalys</t>
+          <t>RSV Data utredning</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Förstudie och kravanalys</t>
+          <t>Utredning av tillgängligt data</t>
         </is>
       </c>
       <c r="D10" s="2">
-        <v>45813</v>
+        <v>45453</v>
       </c>
       <c r="E10" s="2">
-        <v>46203</v>
+        <v>46173</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CUST-LANSA</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>FM-006</t>
+          <t>FM-002</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UPP-010</t>
+          <t>UPP-003</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Baral Azure inloggning</t>
+          <t>Domus automatisering</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Implementering av inloggning Azure Directory</t>
+          <t>Sistemintegration och automatisering</t>
         </is>
       </c>
       <c r="D11" s="2">
-        <v>45935</v>
+        <v>45307</v>
       </c>
       <c r="E11" s="2">
-        <v>46295</v>
+        <v>46203</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>CUST-BARAL</t>
+          <t>CUST-DOMUS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>FM-007</t>
+          <t>FM-001</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>UPP-011</t>
+          <t>UPP-002</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nanometer Datakvalitet</t>
+          <t>Domus Database och BI</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Utredning av datakvalitet</t>
+          <t>Database och BI-mothernisering</t>
         </is>
       </c>
       <c r="D12" s="2">
-        <v>46026</v>
+        <v>45307</v>
       </c>
       <c r="E12" s="2">
         <v>46387</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>CUST-NANOME</t>
+          <t>CUST-DOMUS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>FM-008</t>
+          <t>FM-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>UPP-001</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Domus plattformsmigrering</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Digital plattformsmigrering</t>
+        </is>
+      </c>
+      <c r="D13" s="2">
+        <v>45307</v>
+      </c>
+      <c r="E13" s="2">
+        <v>46173</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CUST-DOMUS</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>FM-001</t>
         </is>
       </c>
     </row>
@@ -3603,7 +3927,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="20.7109375" style="2" customWidth="1"/>
@@ -3655,62 +3979,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TASK-013</t>
+          <t>TASK-014</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nanometer uppgift beslutstöd</t>
+          <t>Postnord uppgift prisprognos</t>
         </is>
       </c>
       <c r="C2" s="2">
         <v>46054</v>
       </c>
       <c r="D2">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E2" s="2">
-        <v>46107</v>
+        <v>46037</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CONS-001</t>
+          <t>CONS-011</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>UPP-011</t>
+          <t>UPP-012</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CUST-NANOME</t>
+          <t>CUST-POSTNO</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TASK-012</t>
+          <t>TASK-013</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nanometer uppgift Cloud utredning</t>
+          <t>Nanometer uppgift beslutstöd</t>
         </is>
       </c>
       <c r="C3" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
       <c r="D3">
-        <v>950</v>
+        <v>1200</v>
       </c>
       <c r="E3" s="2">
-        <v>46107</v>
+        <v>46037</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CONS-008</t>
+          <t>CONS-001</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3727,26 +4051,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TASK-011</t>
+          <t>TASK-012</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nanometer</t>
+          <t>Nanometer uppgift Cloud utredning</t>
         </is>
       </c>
       <c r="C4" s="2">
-        <v>46026</v>
+        <v>46082</v>
       </c>
       <c r="D4">
-        <v>1200</v>
+        <v>950</v>
       </c>
       <c r="E4" s="2">
-        <v>46096</v>
+        <v>46037</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CONS-010</t>
+          <t>CONS-008</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3763,36 +4087,36 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TASK-001</t>
+          <t>TASK-011</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Domus uppgift Platformsmigrering</t>
+          <t>Nanometer</t>
         </is>
       </c>
       <c r="C5" s="2">
-        <v>45307</v>
+        <v>46026</v>
       </c>
       <c r="D5">
         <v>1200</v>
       </c>
       <c r="E5" s="2">
-        <v>46096</v>
+        <v>46037</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CONS-003</t>
+          <t>CONS-010</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>UPP-001</t>
+          <t>UPP-011</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-NANOME</t>
         </is>
       </c>
     </row>
@@ -4115,6 +4439,42 @@
         </is>
       </c>
       <c r="H14" t="inlineStr">
+        <is>
+          <t>CUST-DOMUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TASK-001</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Domus uppgift Platformsmigrering</t>
+        </is>
+      </c>
+      <c r="C15" s="2">
+        <v>45307</v>
+      </c>
+      <c r="D15">
+        <v>1200</v>
+      </c>
+      <c r="E15" s="2">
+        <v>46096</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>CONS-003</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>UPP-001</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>CUST-DOMUS</t>
         </is>
@@ -4127,7 +4487,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="20.7109375" style="2" customWidth="1"/>
@@ -4185,11 +4545,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TR-051</t>
+          <t>TR-052</t>
         </is>
       </c>
       <c r="B2">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="C2" s="2">
         <v>46054</v>
@@ -4202,33 +4562,33 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TASK-011</t>
+          <t>TASK-014</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CONS-010</t>
+          <t>CONS-011</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>UPP-011</t>
+          <t>UPP-012</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CUST-NANOME</t>
+          <t>CUST-POSTNO</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TR-050</t>
+          <t>TR-051</t>
         </is>
       </c>
       <c r="B3">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C3" s="2">
         <v>46054</v>
@@ -4241,33 +4601,33 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TASK-010</t>
+          <t>TASK-011</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CONS-009</t>
+          <t>CONS-010</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>UPP-010</t>
+          <t>UPP-011</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>CUST-BARAL</t>
+          <t>CUST-NANOME</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TR-049</t>
+          <t>TR-050</t>
         </is>
       </c>
       <c r="B4">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="C4" s="2">
         <v>46054</v>
@@ -4280,33 +4640,33 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TASK-009</t>
+          <t>TASK-010</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CONS-008</t>
+          <t>CONS-009</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>UPP-009</t>
+          <t>UPP-010</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>CUST-LANSA</t>
+          <t>CUST-BARAL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TR-048</t>
+          <t>TR-049</t>
         </is>
       </c>
       <c r="B5">
-        <v>61</v>
+        <v>136</v>
       </c>
       <c r="C5" s="2">
         <v>46054</v>
@@ -4319,33 +4679,33 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TASK-008</t>
+          <t>TASK-009</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-008</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>UPP-008</t>
+          <t>UPP-009</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CUST-MONDO</t>
+          <t>CUST-LANSA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TR-047</t>
+          <t>TR-048</t>
         </is>
       </c>
       <c r="B6">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2">
         <v>46054</v>
@@ -4358,33 +4718,33 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TASK-007</t>
+          <t>TASK-008</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CONS-006</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>UPP-007</t>
+          <t>UPP-008</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>CUST-OPUS</t>
+          <t>CUST-MONDO</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TR-046</t>
+          <t>TR-047</t>
         </is>
       </c>
       <c r="B7">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C7" s="2">
         <v>46054</v>
@@ -4397,33 +4757,33 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TASK-006</t>
+          <t>TASK-007</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-006</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>UPP-006</t>
+          <t>UPP-007</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-OPUS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TR-045</t>
+          <t>TR-046</t>
         </is>
       </c>
       <c r="B8">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="C8" s="2">
         <v>46054</v>
@@ -4436,33 +4796,33 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TASK-005</t>
+          <t>TASK-006</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CONS-005</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>UPP-005</t>
+          <t>UPP-006</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>CUST-AVISTA</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TR-044</t>
+          <t>TR-045</t>
         </is>
       </c>
       <c r="B9">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="C9" s="2">
         <v>46054</v>
@@ -4475,33 +4835,33 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TASK-004</t>
+          <t>TASK-005</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>CONS-004</t>
+          <t>CONS-005</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>UPP-004</t>
+          <t>UPP-005</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-AVISTA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TR-043</t>
+          <t>TR-044</t>
         </is>
       </c>
       <c r="B10">
-        <v>120</v>
+        <v>152</v>
       </c>
       <c r="C10" s="2">
         <v>46054</v>
@@ -4514,33 +4874,33 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TASK-003</t>
+          <t>TASK-004</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>CONS-002</t>
+          <t>CONS-004</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>UPP-002</t>
+          <t>UPP-004</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TR-042</t>
+          <t>TR-043</t>
         </is>
       </c>
       <c r="B11">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C11" s="2">
         <v>46054</v>
@@ -4553,17 +4913,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TASK-002</t>
+          <t>TASK-003</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CONS-001</t>
+          <t>CONS-002</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>UPP-003</t>
+          <t>UPP-002</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4575,11 +4935,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TR-041</t>
+          <t>TR-042</t>
         </is>
       </c>
       <c r="B12">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="C12" s="2">
         <v>46054</v>
@@ -4592,17 +4952,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TASK-001</t>
+          <t>TASK-002</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>CONS-003</t>
+          <t>CONS-001</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>UPP-001</t>
+          <t>UPP-003</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4614,50 +4974,50 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TR-040</t>
+          <t>TR-041</t>
         </is>
       </c>
       <c r="B13">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="C13" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="D13" s="2">
-        <v>46053</v>
+        <v>46081</v>
       </c>
       <c r="E13" s="2">
-        <v>46068</v>
+        <v>46096</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TASK-011</t>
+          <t>TASK-001</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>CONS-010</t>
+          <t>CONS-003</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>UPP-011</t>
+          <t>UPP-001</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>CUST-NANOME</t>
+          <t>CUST-DOMUS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TR-039</t>
+          <t>TR-040</t>
         </is>
       </c>
       <c r="B14">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C14" s="2">
         <v>46023</v>
@@ -4670,33 +5030,33 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TASK-010</t>
+          <t>TASK-011</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CONS-009</t>
+          <t>CONS-010</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>UPP-010</t>
+          <t>UPP-011</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>CUST-BARAL</t>
+          <t>CUST-NANOME</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TR-038</t>
+          <t>TR-039</t>
         </is>
       </c>
       <c r="B15">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C15" s="2">
         <v>46023</v>
@@ -4709,33 +5069,33 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TASK-009</t>
+          <t>TASK-010</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CONS-008</t>
+          <t>CONS-009</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>UPP-009</t>
+          <t>UPP-010</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>CUST-LANSA</t>
+          <t>CUST-BARAL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TR-037</t>
+          <t>TR-038</t>
         </is>
       </c>
       <c r="B16">
-        <v>50</v>
+        <v>136</v>
       </c>
       <c r="C16" s="2">
         <v>46023</v>
@@ -4748,33 +5108,33 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TASK-008</t>
+          <t>TASK-009</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-008</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>UPP-008</t>
+          <t>UPP-009</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>CUST-MONDO</t>
+          <t>CUST-LANSA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TR-036</t>
+          <t>TR-037</t>
         </is>
       </c>
       <c r="B17">
-        <v>160</v>
+        <v>50</v>
       </c>
       <c r="C17" s="2">
         <v>46023</v>
@@ -4787,33 +5147,33 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TASK-007</t>
+          <t>TASK-008</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CONS-006</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>UPP-007</t>
+          <t>UPP-008</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>CUST-OPUS</t>
+          <t>CUST-MONDO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TR-035</t>
+          <t>TR-036</t>
         </is>
       </c>
       <c r="B18">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="C18" s="2">
         <v>46023</v>
@@ -4826,33 +5186,33 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TASK-006</t>
+          <t>TASK-007</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-006</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>UPP-006</t>
+          <t>UPP-007</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-OPUS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TR-034</t>
+          <t>TR-035</t>
         </is>
       </c>
       <c r="B19">
-        <v>158</v>
+        <v>80</v>
       </c>
       <c r="C19" s="2">
         <v>46023</v>
@@ -4865,33 +5225,33 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TASK-005</t>
+          <t>TASK-006</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CONS-005</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>UPP-005</t>
+          <t>UPP-006</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>CUST-AVISTA</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TR-033</t>
+          <t>TR-034</t>
         </is>
       </c>
       <c r="B20">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C20" s="2">
         <v>46023</v>
@@ -4904,33 +5264,33 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TASK-004</t>
+          <t>TASK-005</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CONS-004</t>
+          <t>CONS-005</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>UPP-004</t>
+          <t>UPP-005</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-AVISTA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TR-032</t>
+          <t>TR-033</t>
         </is>
       </c>
       <c r="B21">
-        <v>115</v>
+        <v>155</v>
       </c>
       <c r="C21" s="2">
         <v>46023</v>
@@ -4943,33 +5303,33 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TASK-003</t>
+          <t>TASK-004</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CONS-002</t>
+          <t>CONS-004</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>UPP-002</t>
+          <t>UPP-004</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TR-031</t>
+          <t>TR-032</t>
         </is>
       </c>
       <c r="B22">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="C22" s="2">
         <v>46023</v>
@@ -4982,17 +5342,17 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TASK-002</t>
+          <t>TASK-003</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>CONS-001</t>
+          <t>CONS-002</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>UPP-003</t>
+          <t>UPP-002</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5004,11 +5364,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TR-030</t>
+          <t>TR-031</t>
         </is>
       </c>
       <c r="B23">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="C23" s="2">
         <v>46023</v>
@@ -5021,17 +5381,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>TASK-001</t>
+          <t>TASK-002</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>CONS-003</t>
+          <t>CONS-001</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>UPP-001</t>
+          <t>UPP-003</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5043,50 +5403,50 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TR-029</t>
+          <t>TR-030</t>
         </is>
       </c>
       <c r="B24">
-        <v>114</v>
+        <v>156</v>
       </c>
       <c r="C24" s="2">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="D24" s="2">
-        <v>46022</v>
+        <v>46053</v>
       </c>
       <c r="E24" s="2">
-        <v>46037</v>
+        <v>46068</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>TASK-010</t>
+          <t>TASK-001</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>CONS-009</t>
+          <t>CONS-003</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>UPP-010</t>
+          <t>UPP-001</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>CUST-BARAL</t>
+          <t>CUST-DOMUS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TR-028</t>
+          <t>TR-029</t>
         </is>
       </c>
       <c r="B25">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="C25" s="2">
         <v>45992</v>
@@ -5099,33 +5459,33 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>TASK-009</t>
+          <t>TASK-010</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>CONS-008</t>
+          <t>CONS-009</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>UPP-009</t>
+          <t>UPP-010</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CUST-LANSA</t>
+          <t>CUST-BARAL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TR-027</t>
+          <t>TR-028</t>
         </is>
       </c>
       <c r="B26">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="C26" s="2">
         <v>45992</v>
@@ -5138,33 +5498,33 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>TASK-008</t>
+          <t>TASK-009</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-008</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>UPP-008</t>
+          <t>UPP-009</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>CUST-MONDO</t>
+          <t>CUST-LANSA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TR-026</t>
+          <t>TR-027</t>
         </is>
       </c>
       <c r="B27">
-        <v>152</v>
+        <v>60</v>
       </c>
       <c r="C27" s="2">
         <v>45992</v>
@@ -5177,33 +5537,33 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>TASK-007</t>
+          <t>TASK-008</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>CONS-006</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>UPP-007</t>
+          <t>UPP-008</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CUST-OPUS</t>
+          <t>CUST-MONDO</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TR-025</t>
+          <t>TR-026</t>
         </is>
       </c>
       <c r="B28">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="C28" s="2">
         <v>45992</v>
@@ -5216,33 +5576,33 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TASK-006</t>
+          <t>TASK-007</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-006</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>UPP-006</t>
+          <t>UPP-007</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-OPUS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TR-024</t>
+          <t>TR-025</t>
         </is>
       </c>
       <c r="B29">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="C29" s="2">
         <v>45992</v>
@@ -5255,33 +5615,33 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>TASK-005</t>
+          <t>TASK-006</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>CONS-005</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>UPP-005</t>
+          <t>UPP-006</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>CUST-AVISTA</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TR-023</t>
+          <t>TR-024</t>
         </is>
       </c>
       <c r="B30">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C30" s="2">
         <v>45992</v>
@@ -5294,33 +5654,33 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>TASK-004</t>
+          <t>TASK-005</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>CONS-004</t>
+          <t>CONS-005</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>UPP-004</t>
+          <t>UPP-005</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-AVISTA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TR-022</t>
+          <t>TR-023</t>
         </is>
       </c>
       <c r="B31">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="C31" s="2">
         <v>45992</v>
@@ -5333,33 +5693,33 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>TASK-003</t>
+          <t>TASK-004</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>CONS-002</t>
+          <t>CONS-004</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>UPP-002</t>
+          <t>UPP-004</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TR-021</t>
+          <t>TR-022</t>
         </is>
       </c>
       <c r="B32">
-        <v>76</v>
+        <v>114</v>
       </c>
       <c r="C32" s="2">
         <v>45992</v>
@@ -5372,17 +5732,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TASK-002</t>
+          <t>TASK-003</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>CONS-001</t>
+          <t>CONS-002</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>UPP-003</t>
+          <t>UPP-002</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -5394,11 +5754,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TR-020</t>
+          <t>TR-021</t>
         </is>
       </c>
       <c r="B33">
-        <v>150</v>
+        <v>76</v>
       </c>
       <c r="C33" s="2">
         <v>45992</v>
@@ -5411,17 +5771,17 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>TASK-001</t>
+          <t>TASK-002</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>CONS-003</t>
+          <t>CONS-001</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>UPP-001</t>
+          <t>UPP-003</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -5433,50 +5793,50 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TR-019</t>
+          <t>TR-020</t>
         </is>
       </c>
       <c r="B34">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="C34" s="2">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="D34" s="2">
-        <v>45991</v>
+        <v>46022</v>
       </c>
       <c r="E34" s="2">
-        <v>46006</v>
+        <v>46037</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>TASK-010</t>
+          <t>TASK-001</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>CONS-009</t>
+          <t>CONS-003</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>UPP-010</t>
+          <t>UPP-001</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>CUST-BARAL</t>
+          <t>CUST-DOMUS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TR-018</t>
+          <t>TR-019</t>
         </is>
       </c>
       <c r="B35">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C35" s="2">
         <v>45962</v>
@@ -5489,33 +5849,33 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>TASK-009</t>
+          <t>TASK-010</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>CONS-008</t>
+          <t>CONS-009</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>UPP-009</t>
+          <t>UPP-010</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>CUST-LANSA</t>
+          <t>CUST-BARAL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TR-017</t>
+          <t>TR-018</t>
         </is>
       </c>
       <c r="B36">
-        <v>70</v>
+        <v>135</v>
       </c>
       <c r="C36" s="2">
         <v>45962</v>
@@ -5528,33 +5888,33 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>TASK-008</t>
+          <t>TASK-009</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-008</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>UPP-008</t>
+          <t>UPP-009</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>CUST-MONDO</t>
+          <t>CUST-LANSA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TR-016</t>
+          <t>TR-017</t>
         </is>
       </c>
       <c r="B37">
-        <v>154</v>
+        <v>70</v>
       </c>
       <c r="C37" s="2">
         <v>45962</v>
@@ -5567,33 +5927,33 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>TASK-007</t>
+          <t>TASK-008</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>CONS-006</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>UPP-007</t>
+          <t>UPP-008</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>CUST-OPUS</t>
+          <t>CUST-MONDO</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TR-015</t>
+          <t>TR-016</t>
         </is>
       </c>
       <c r="B38">
-        <v>78</v>
+        <v>154</v>
       </c>
       <c r="C38" s="2">
         <v>45962</v>
@@ -5606,33 +5966,33 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>TASK-006</t>
+          <t>TASK-007</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-006</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>UPP-006</t>
+          <t>UPP-007</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-OPUS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TR-014</t>
+          <t>TR-015</t>
         </is>
       </c>
       <c r="B39">
-        <v>168</v>
+        <v>78</v>
       </c>
       <c r="C39" s="2">
         <v>45962</v>
@@ -5645,33 +6005,33 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>TASK-005</t>
+          <t>TASK-006</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>CONS-005</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>UPP-005</t>
+          <t>UPP-006</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>CUST-AVISTA</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TR-013</t>
+          <t>TR-014</t>
         </is>
       </c>
       <c r="B40">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C40" s="2">
         <v>45962</v>
@@ -5684,33 +6044,33 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>TASK-004</t>
+          <t>TASK-005</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>CONS-004</t>
+          <t>CONS-005</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>UPP-004</t>
+          <t>UPP-005</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-AVISTA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TR-012</t>
+          <t>TR-013</t>
         </is>
       </c>
       <c r="B41">
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="C41" s="2">
         <v>45962</v>
@@ -5723,33 +6083,33 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>TASK-003</t>
+          <t>TASK-004</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>CONS-002</t>
+          <t>CONS-004</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>UPP-002</t>
+          <t>UPP-004</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TR-011</t>
+          <t>TR-012</t>
         </is>
       </c>
       <c r="B42">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="C42" s="2">
         <v>45962</v>
@@ -5762,17 +6122,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>TASK-002</t>
+          <t>TASK-003</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>CONS-001</t>
+          <t>CONS-002</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>UPP-003</t>
+          <t>UPP-002</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -5784,11 +6144,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TR-010</t>
+          <t>TR-011</t>
         </is>
       </c>
       <c r="B43">
-        <v>160</v>
+        <v>78</v>
       </c>
       <c r="C43" s="2">
         <v>45962</v>
@@ -5801,17 +6161,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>TASK-001</t>
+          <t>TASK-002</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>CONS-003</t>
+          <t>CONS-001</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>UPP-001</t>
+          <t>UPP-003</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -5823,50 +6183,50 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TR-009</t>
+          <t>TR-010</t>
         </is>
       </c>
       <c r="B44">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C44" s="2">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="D44" s="2">
-        <v>45961</v>
+        <v>45991</v>
       </c>
       <c r="E44" s="2">
-        <v>45976</v>
+        <v>46006</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>TASK-009</t>
+          <t>TASK-001</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>CONS-008</t>
+          <t>CONS-003</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>UPP-009</t>
+          <t>UPP-001</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>CUST-LANSA</t>
+          <t>CUST-DOMUS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TR-008</t>
+          <t>TR-009</t>
         </is>
       </c>
       <c r="B45">
-        <v>82</v>
+        <v>147</v>
       </c>
       <c r="C45" s="2">
         <v>45931</v>
@@ -5879,33 +6239,33 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>TASK-008</t>
+          <t>TASK-009</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-008</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>UPP-008</t>
+          <t>UPP-009</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>CUST-MONDO</t>
+          <t>CUST-LANSA</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TR-007</t>
+          <t>TR-008</t>
         </is>
       </c>
       <c r="B46">
-        <v>178</v>
+        <v>82</v>
       </c>
       <c r="C46" s="2">
         <v>45931</v>
@@ -5918,33 +6278,33 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>TASK-007</t>
+          <t>TASK-008</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>CONS-006</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>UPP-007</t>
+          <t>UPP-008</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>CUST-OPUS</t>
+          <t>CUST-MONDO</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TR-006</t>
+          <t>TR-007</t>
         </is>
       </c>
       <c r="B47">
-        <v>92</v>
+        <v>178</v>
       </c>
       <c r="C47" s="2">
         <v>45931</v>
@@ -5957,33 +6317,33 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>TASK-006</t>
+          <t>TASK-007</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>CONS-007</t>
+          <t>CONS-006</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>UPP-006</t>
+          <t>UPP-007</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-OPUS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TR-005</t>
+          <t>TR-006</t>
         </is>
       </c>
       <c r="B48">
-        <v>184</v>
+        <v>92</v>
       </c>
       <c r="C48" s="2">
         <v>45931</v>
@@ -5996,33 +6356,33 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>TASK-005</t>
+          <t>TASK-006</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>CONS-005</t>
+          <t>CONS-007</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>UPP-005</t>
+          <t>UPP-006</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>CUST-AVISTA</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TR-004</t>
+          <t>TR-005</t>
         </is>
       </c>
       <c r="B49">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="C49" s="2">
         <v>45931</v>
@@ -6035,33 +6395,33 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>TASK-004</t>
+          <t>TASK-005</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>CONS-004</t>
+          <t>CONS-005</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>UPP-004</t>
+          <t>UPP-005</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>CUST-RSV</t>
+          <t>CUST-AVISTA</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TR-003</t>
+          <t>TR-004</t>
         </is>
       </c>
       <c r="B50">
-        <v>138</v>
+        <v>177</v>
       </c>
       <c r="C50" s="2">
         <v>45931</v>
@@ -6074,33 +6434,33 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>TASK-003</t>
+          <t>TASK-004</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>CONS-002</t>
+          <t>CONS-004</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>UPP-002</t>
+          <t>UPP-004</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>CUST-DOMUS</t>
+          <t>CUST-RSV</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TR-002</t>
+          <t>TR-003</t>
         </is>
       </c>
       <c r="B51">
-        <v>89</v>
+        <v>138</v>
       </c>
       <c r="C51" s="2">
         <v>45931</v>
@@ -6113,17 +6473,17 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>TASK-002</t>
+          <t>TASK-003</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>CONS-001</t>
+          <t>CONS-002</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>UPP-003</t>
+          <t>UPP-002</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -6135,11 +6495,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TR-001</t>
+          <t>TR-002</t>
         </is>
       </c>
       <c r="B52">
-        <v>180</v>
+        <v>89</v>
       </c>
       <c r="C52" s="2">
         <v>45931</v>
@@ -6152,20 +6512,59 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
+          <t>TASK-002</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>CONS-001</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>UPP-003</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>CUST-DOMUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TR-001</t>
+        </is>
+      </c>
+      <c r="B53">
+        <v>180</v>
+      </c>
+      <c r="C53" s="2">
+        <v>45931</v>
+      </c>
+      <c r="D53" s="2">
+        <v>45961</v>
+      </c>
+      <c r="E53" s="2">
+        <v>45976</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
           <t>TASK-001</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>CONS-003</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>UPP-001</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>CUST-DOMUS</t>
         </is>
@@ -6178,7 +6577,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -7145,6 +7544,39 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TP-029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>UPP-012</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TASK-014</t>
+        </is>
+      </c>
+      <c r="E30">
+        <v>1100</v>
+      </c>
+      <c r="F30" s="2">
+        <v>46037</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Auto från Uppgift-formulär</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7152,7 +7584,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
@@ -7676,6 +8108,52 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GL-023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="C24">
+        <v>50000</v>
+      </c>
+      <c r="D24" s="2">
+        <v>46054</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Auto vid ny konsult</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GL-024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CONS-011</t>
+        </is>
+      </c>
+      <c r="C25">
+        <v>52000</v>
+      </c>
+      <c r="D25" s="2">
+        <v>46054</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Auto: ändring grundlon i Konsulter-tabell</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>